<commit_message>
fix(i18n): owner-reviewed EN dictionary + fix 2 RU label typos in source xlsx
- EN overlay reviewed by owner → enTranslationStatus "owner-reviewed"
  (translations.en.json value polish + _note; etl.py status flip)
- Source workbook had 2 RU label typos surfaced by the review; fixed in
  xl/sharedStrings.xml via surgical zip edit (cached <v> untouched), so the
  reviewed EN keys match the source again:
    "проивзодства"→"производства" (Расчёты!C211,C248)
    "Тепловая мощности ТЭЦ"→"…мощность…" (Расчёты!C148)
  → modelVersion kz-4c2d4a8b30a3 (hash bump only; data/calc unchanged:
    abatement 214,353 kt, wavg MAC 95.6, no-regrets 12,610), golden 188/188,
    0 empty EN labels, build green (First Load 178 kB)
- RU UI: onboarding "меры «без сожалений»" → "меры «no-regret»" (matches the
  established term already used in kpi/table badges)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MACC_KZ_29052026_rev.xlsx
+++ b/MACC_KZ_29052026_rev.xlsx
@@ -963,7 +963,7 @@
     <t>Паровая+водогрейная котельная</t>
   </si>
   <si>
-    <t>Тепловая мощности ТЭЦ</t>
+    <t>Тепловая мощность ТЭЦ</t>
   </si>
   <si>
     <t>выработк</t>
@@ -1029,7 +1029,7 @@
     <t>[1.A.1-6] Тепловые насосы для централизованного теплоснабжения</t>
   </si>
   <si>
-    <t>Общий объем проивзодства тепла</t>
+    <t>Общий объем производства тепла</t>
   </si>
   <si>
     <t>тыс Гкал</t>

</xml_diff>